<commit_message>
Enhance ConceptMap with additional mappings and descriptions
Updated the ConceptMap to include additional mappings and descriptions for CDA CE, CS, and CD datatypes to FHIR code, CodeableConcept, and Coding. Adjusted display names and comments for clarity. 2d934d41d8b353373de2725b070f099b3a099d9d
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaCECSCDToCodeConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaCECSCDToCodeConceptMap.xlsx
@@ -13,12 +13,14 @@
     <sheet name="Mapping Table 3" r:id="rId7" sheetId="5"/>
     <sheet name="Mapping Table 4" r:id="rId8" sheetId="6"/>
     <sheet name="Mapping Table 5" r:id="rId9" sheetId="7"/>
+    <sheet name="Mapping Table 6" r:id="rId10" sheetId="8"/>
+    <sheet name="Mapping Table 7" r:id="rId11" sheetId="9"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="67">
   <si>
     <t>Property</t>
   </si>
@@ -29,7 +31,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaConceptCodesToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaCECSCDToCodeConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -65,7 +67,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T12:41:23+00:00</t>
+    <t>2026-07-22T12:48:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -89,7 +91,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Correspondances documentaires entre les datatypes CDA CE, CS et CD et les types FHIR code et CodeableConcept.</t>
+    <t>Correspondances documentaires entre les datatypes CDA CE, CS et CD et les types FHIR code, CodeableConcept et Coding.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -122,46 +124,79 @@
     <t>CE.code</t>
   </si>
   <si>
+    <t>Code</t>
+  </si>
+  <si>
     <t>equivalent</t>
   </si>
   <si>
     <t>code</t>
   </si>
   <si>
+    <t>Primitive Type code</t>
+  </si>
+  <si>
     <t>http://hl7.org/fhir/StructureDefinition/CodeableConcept|4.0.1</t>
   </si>
   <si>
     <t>CE.originalText</t>
   </si>
   <si>
+    <t>Original Text</t>
+  </si>
+  <si>
     <t>CodeableConcept.text</t>
   </si>
   <si>
-    <t>CodeableConcept.coding.code</t>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>CE.translation</t>
+  </si>
+  <si>
+    <t>Translation</t>
+  </si>
+  <si>
+    <t>related-to</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/StructureDefinition/Coding|4.0.1</t>
+  </si>
+  <si>
+    <t>Coding.code</t>
+  </si>
+  <si>
+    <t>Symbol in syntax defined by the system</t>
   </si>
   <si>
     <t>CE.codeSystem</t>
   </si>
   <si>
-    <t>related-to</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding.system</t>
+    <t>Code System</t>
+  </si>
+  <si>
+    <t>Coding.system</t>
+  </si>
+  <si>
+    <t>Identity of the terminology system</t>
   </si>
   <si>
     <t>CE.displayName</t>
   </si>
   <si>
-    <t>CodeableConcept.coding.display</t>
-  </si>
-  <si>
-    <t>CE.translation</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding (translation)</t>
+    <t>Display Name</t>
+  </si>
+  <si>
+    <t>Coding.display</t>
+  </si>
+  <si>
+    <t>Representation defined by the system</t>
   </si>
   <si>
     <t>http://hl7.org/cda/stds/core/StructureDefinition/CS|2.0.0-sd</t>
@@ -179,13 +214,13 @@
     <t>CD.originalText</t>
   </si>
   <si>
+    <t>CD.translation</t>
+  </si>
+  <si>
     <t>CD.codeSystem</t>
   </si>
   <si>
     <t>CD.displayName</t>
-  </si>
-  <si>
-    <t>CD.translation</t>
   </si>
 </sst>
 </file>
@@ -483,16 +518,16 @@
         <v>33</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -502,7 +537,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -533,7 +568,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -541,86 +576,35 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B5" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D5" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="E5" t="s" s="2">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="B6" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="C6" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D6" t="s" s="2">
-        <v>44</v>
-      </c>
-      <c r="E6" t="s" s="2">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="B7" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D7" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="E7" t="s" s="2">
         <v>47</v>
       </c>
     </row>
@@ -631,7 +615,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -653,16 +637,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
         <v>48</v>
-      </c>
-      <c r="B2" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="C2" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="D2" t="s" s="2">
-        <v>32</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -670,19 +654,53 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="D3" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="B3" t="s" s="2">
-        <v>49</v>
-      </c>
-      <c r="C3" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D3" t="s" s="2">
+      <c r="E3" t="s" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s" s="2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>56</v>
+      </c>
+      <c r="C5" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="E3" t="s" s="2">
-        <v>35</v>
+      <c r="D5" t="s" s="2">
+        <v>57</v>
+      </c>
+      <c r="E5" t="s" s="2">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -714,7 +732,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -723,7 +741,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -731,19 +749,19 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -775,7 +793,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -784,7 +802,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -792,19 +810,19 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -814,7 +832,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -836,7 +854,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -845,7 +863,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -853,87 +871,192 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="E2" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>63</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D3" t="s" s="2">
-        <v>38</v>
-      </c>
       <c r="E3" t="s" s="2">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>39</v>
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="E2" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>65</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s" s="2">
+        <v>54</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="B6" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="C6" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D6" t="s" s="2">
-        <v>44</v>
-      </c>
-      <c r="E6" t="s" s="2">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="2">
-        <v>55</v>
-      </c>
-      <c r="B7" t="s" s="2">
-        <v>55</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D7" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="E7" t="s" s="2">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>